<commit_message>
chore(templates): regenerate standardized Excel templates with closed reference graph
</commit_message>
<xml_diff>
--- a/templates/HEADWAY_INFRASTRUCTURE_v1.0.xlsx
+++ b/templates/HEADWAY_INFRASTRUCTURE_v1.0.xlsx
@@ -567,7 +567,7 @@
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>3. Row 3 contains an illustrative example row (marked with ID 'EXAMPLE_*'). Replace or delete before production use.</t>
+          <t>3. Row 3 contains a minimal valid baseline network for demonstration purposes. You may modify or replace it with your own railway data. The example is designed to load without validation errors.</t>
         </is>
       </c>
     </row>
@@ -889,7 +889,7 @@
       </c>
       <c r="C3" s="10" t="inlineStr">
         <is>
-          <t>BLK_01, BLK_02</t>
+          <t>BLK_01</t>
         </is>
       </c>
     </row>
@@ -1018,7 +1018,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:C4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1074,6 +1074,23 @@
       <c r="C3" s="10" t="inlineStr">
         <is>
           <t>BUFFER_STOP</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="10" t="inlineStr">
+        <is>
+          <t>ND_02</t>
+        </is>
+      </c>
+      <c r="B4" s="10" t="inlineStr">
+        <is>
+          <t>Downstream endpoint</t>
+        </is>
+      </c>
+      <c r="C4" s="10" t="inlineStr">
+        <is>
+          <t>ENDPOINT</t>
         </is>
       </c>
     </row>

</xml_diff>